<commit_message>
Excel Builder Block14 Proposal and Trace Sheets
</commit_message>
<xml_diff>
--- a/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
+++ b/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxepunkter" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sammanfattning" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa_Förslag" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelspårning" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxepunkter'!$A$1:$J$242</definedName>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +34,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +50,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,12 +75,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -154,6 +179,45 @@
     <tableColumn id="8" name="EDP koppling status"/>
     <tableColumn id="9" name="Kommentar"/>
     <tableColumn id="10" name="Källa"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TaxaForslagTable" displayName="TaxaForslagTable" ref="A6:K7" headerRowCount="1">
+  <autoFilter ref="A6:K7"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="Kommun"/>
+    <tableColumn id="2" name="Paragraf"/>
+    <tableColumn id="3" name="Taxapunkt"/>
+    <tableColumn id="4" name="Variant"/>
+    <tableColumn id="5" name="Enhet"/>
+    <tableColumn id="6" name="Föreslagen taxekod"/>
+    <tableColumn id="7" name="Föreslagen benämning"/>
+    <tableColumn id="8" name="Källa"/>
+    <tableColumn id="9" name="Säkerhet"/>
+    <tableColumn id="10" name="Status"/>
+    <tableColumn id="11" name="Kommentar"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RegelsparningTable" displayName="RegelsparningTable" ref="A6:J7" headerRowCount="1">
+  <autoFilter ref="A6:J7"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Kommun"/>
+    <tableColumn id="2" name="Paragraf"/>
+    <tableColumn id="3" name="Taxapunkt"/>
+    <tableColumn id="4" name="Fält"/>
+    <tableColumn id="5" name="Värde"/>
+    <tableColumn id="6" name="Ursprung"/>
+    <tableColumn id="7" name="Regel"/>
+    <tableColumn id="8" name="Källa"/>
+    <tableColumn id="9" name="Status"/>
+    <tableColumn id="10" name="Kommentar"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8818,7 +8882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -8866,6 +8930,30 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>Arbets-Excel – inte master</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Taxa_Förslag</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ingår för föreslagna saknade taxekoder</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Regelspårning</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ingår för spårbarhet</t>
         </is>
       </c>
     </row>
@@ -8880,7 +8968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -8889,7 +8977,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Excel Builder v2.0.0-alpha.1</t>
+          <t>Excel Builder</t>
         </is>
       </c>
     </row>
@@ -8916,33 +9004,43 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nästa steg:</t>
+          <t>Taxa_Förslag och Regelspårning ingår i alla genererade arbetsböcker.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1. Koppla mot befintlig Arbets-Excel/EDP-data.</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2. Behåll befintliga EDP-koder där matchning är säker.</t>
+          <t>Nästa steg:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3. Markera osäkra rader för manuell kontroll.</t>
+          <t>1. Koppla mot befintlig Arbets-Excel/EDP-data.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>2. Behåll befintliga EDP-koder där matchning är säker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3. Markera osäkra rader för manuell kontroll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>4. Skapa ny godkänd arbetsversion.</t>
         </is>
@@ -8951,4 +9049,311 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Taxa_Förslag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Syfte</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Förslag på saknade taxekoder. Förslag ska granskas innan import till EDP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Källa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Parseroutput</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Paragraf</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Taxapunkt</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Enhet</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Föreslagen taxekod</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Föreslagen benämning</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Källa</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Säkerhet</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>EDP Standardtaxor / regelverk / manuell granskning</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Ej granskad</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>EDP-data får aldrig blandas mellan projekt.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Regelspårning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Syfte</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Spårar hur varje rad/fält byggdes: Word, EDP, standardtaxor eller manuell granskning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Källa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Parseroutput</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Paragraf</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Taxapunkt</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Fält</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Värde</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Ursprung</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Regel</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Källa</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Kommentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Taxakod</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Ej satt</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Taxakod får endast sättas från säker EDP-match eller markerat förslag.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Regelverk</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Ej granskad</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Standardflik för framtida spårning.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel Builder Block15.1 Standard Tax ZIP and Fixed EDP Rule
</commit_message>
<xml_diff>
--- a/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
+++ b/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sammanfattning" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxa_Förslag" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelspårning" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDP_Avviker_Standard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regelspårning" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Taxepunkter'!$A$1:$J$242</definedName>
@@ -205,7 +206,28 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RegelsparningTable" displayName="RegelsparningTable" ref="A6:J7" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EdpAvvikerStandardTable" displayName="EdpAvvikerStandardTable" ref="A6:L7" headerRowCount="1">
+  <autoFilter ref="A6:L7"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Kommun"/>
+    <tableColumn id="2" name="EDP taxekod"/>
+    <tableColumn id="3" name="EDP benämning"/>
+    <tableColumn id="4" name="EDP faktor"/>
+    <tableColumn id="5" name="EDP taxedel"/>
+    <tableColumn id="6" name="Standard taxekod"/>
+    <tableColumn id="7" name="Standard benämning"/>
+    <tableColumn id="8" name="Standard faktor"/>
+    <tableColumn id="9" name="Standard taxedel"/>
+    <tableColumn id="10" name="Avvikelse"/>
+    <tableColumn id="11" name="Rekommendation"/>
+    <tableColumn id="12" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RegelsparningTable" displayName="RegelsparningTable" ref="A6:J7" headerRowCount="1">
   <autoFilter ref="A6:J7"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Kommun"/>
@@ -9208,6 +9230,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="54" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>EDP Export avviker från standardtaxa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Syfte</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Visar avvikelser mot standardtaxor. Befintlig Taxa_från_edp är fast och ändras aldrig automatiskt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Källa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Parseroutput</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Kommun</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>EDP taxekod</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>EDP benämning</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>EDP faktor</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>EDP taxedel</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Standard taxekod</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Standard benämning</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Standard faktor</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Standard taxedel</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Avvikelse</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>Rekommendation</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>Granska manuellt. Ändra inte befintlig EDP automatiskt.</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Ej granskad</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9217,7 +9393,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
@@ -9331,7 +9507,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Taxakod får endast sättas från säker EDP-match eller markerat förslag.</t>
+          <t>Befintlig Taxa_från_edp är fast. Standardtaxor får endast ge förslag/avvikelse.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Excel Builder Block20.3 Knowledge Token and Project Scope Fix
</commit_message>
<xml_diff>
--- a/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
+++ b/output/excel/ArbetsExcel_byggd_fran_parser.xlsx
@@ -23784,7 +23784,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>tvåbostadshus</t>
+          <t>en-och, tvåbostadshus</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -24097,7 +24097,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>campingstuga, lägenhet</t>
+          <t>-lägenhet, campingstuga, lägenhet</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
@@ -24160,7 +24160,7 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>240, kärl, mat, restavfall</t>
+          <t>240, kärl, mat-, restavfall</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr"/>
@@ -24190,7 +24190,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Träavfall</t>
+          <t>Restavfall</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -24274,7 +24274,7 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>240, kärl, mat, restavfall</t>
+          <t>240, kärl, mat-, restavfall</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr"/>
@@ -24304,7 +24304,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Träavfall</t>
+          <t>Restavfall</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -24372,7 +24372,7 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>gemensam, mat, restavfall, uppsamlingsplats</t>
+          <t>gemensam, mat-, restavfall, uppsamlingsplats</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
@@ -24404,17 +24404,13 @@
           <t>Hushåll</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -24424,7 +24420,7 @@
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -24452,20 +24448,12 @@
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>Tillfälle</t>
-        </is>
-      </c>
+      <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>TILLFÄLLE</t>
-        </is>
-      </c>
+      <c r="J20" s="6" t="inlineStr"/>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -24475,7 +24463,7 @@
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>Avfallstyp kunde inte härledas.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -24619,7 +24607,7 @@
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>240, kärl, mat, restavfall</t>
+          <t>240, kärl, mat-, restavfall</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr"/>
@@ -25134,7 +25122,7 @@
       </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
-          <t>förpackningar, mat, restavfall</t>
+          <t>förpackningar, mat-, restavfall</t>
         </is>
       </c>
       <c r="M32" s="6" t="inlineStr">
@@ -25197,7 +25185,7 @@
       </c>
       <c r="L33" s="6" t="inlineStr">
         <is>
-          <t>240, kärl, mat, restavfall</t>
+          <t>240, kärl, mat-, restavfall</t>
         </is>
       </c>
       <c r="M33" s="6" t="inlineStr"/>
@@ -25417,7 +25405,7 @@
       </c>
       <c r="L37" s="6" t="inlineStr">
         <is>
-          <t>behållare, bottentömmande, mat, restavfall</t>
+          <t>behållare, bottentömmande, mat-, restavfall</t>
         </is>
       </c>
       <c r="M37" s="6" t="inlineStr">
@@ -25527,7 +25515,7 @@
       </c>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>240, kärl, mat, restavfall</t>
+          <t>240, kärl, mat-, restavfall</t>
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr"/>
@@ -25747,7 +25735,7 @@
       </c>
       <c r="L43" s="6" t="inlineStr">
         <is>
-          <t>behållare, bottentömmande, mat, restavfall</t>
+          <t>behållare, bottentömmande, mat-, restavfall</t>
         </is>
       </c>
       <c r="M43" s="6" t="inlineStr">
@@ -25853,7 +25841,7 @@
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
-          <t>140, kontors, kärl, returpapper</t>
+          <t>140, kontors-, kärl, returpapper</t>
         </is>
       </c>
       <c r="M45" s="6" t="inlineStr">
@@ -25896,7 +25884,7 @@
       </c>
       <c r="L46" s="6" t="inlineStr">
         <is>
-          <t>anvisning, egen, enligt, förbrukat, kontors, returpapper, överlämning</t>
+          <t>anvisning, egen, enligt, förbrukat, kontors-, returpapper, överlämning</t>
         </is>
       </c>
       <c r="M46" s="6" t="inlineStr">
@@ -26279,7 +26267,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Träavfall</t>
+          <t>Matavfall</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
@@ -26338,7 +26326,7 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Träavfall</t>
+          <t>Restavfall</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
@@ -26363,7 +26351,7 @@
       </c>
       <c r="L55" s="6" t="inlineStr">
         <is>
-          <t>140, 190, extra, kilogram, kärl, restavfall</t>
+          <t>140-190, extra, kilogram, kärl, restavfall</t>
         </is>
       </c>
       <c r="M55" s="6" t="inlineStr"/>
@@ -26603,17 +26591,13 @@
           <t>Hushåll</t>
         </is>
       </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G60" s="6" t="inlineStr"/>
       <c r="H60" s="6" t="inlineStr"/>
       <c r="I60" s="6" t="inlineStr"/>
       <c r="J60" s="6" t="inlineStr"/>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr">
@@ -26623,7 +26607,7 @@
       </c>
       <c r="M60" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -26677,7 +26661,7 @@
       </c>
       <c r="L61" s="6" t="inlineStr">
         <is>
-          <t>140, 240, byte, ggr, kärl, liter, återtag</t>
+          <t>140-240, byte, ggr, kärl, liter, återtag</t>
         </is>
       </c>
       <c r="M61" s="6" t="inlineStr">
@@ -26736,7 +26720,7 @@
       </c>
       <c r="L62" s="6" t="inlineStr">
         <is>
-          <t>370, 660, byte, ggr, kärl, liter, återtag</t>
+          <t>370-660, byte, ggr, kärl, liter, återtag</t>
         </is>
       </c>
       <c r="M62" s="6" t="inlineStr">
@@ -26932,7 +26916,7 @@
       </c>
       <c r="L66" s="6" t="inlineStr">
         <is>
-          <t>140, 660, kärl</t>
+          <t>140-660, 5-10, kärl</t>
         </is>
       </c>
       <c r="M66" s="6" t="inlineStr">
@@ -26991,7 +26975,7 @@
       </c>
       <c r="L67" s="6" t="inlineStr">
         <is>
-          <t>140, 660, kärl</t>
+          <t>10-20, 140-660, kärl</t>
         </is>
       </c>
       <c r="M67" s="6" t="inlineStr">
@@ -27050,7 +27034,7 @@
       </c>
       <c r="L68" s="6" t="inlineStr">
         <is>
-          <t>140, 660, kärl</t>
+          <t>140-660, 20-30, kärl</t>
         </is>
       </c>
       <c r="M68" s="6" t="inlineStr">
@@ -27662,11 +27646,7 @@
           <t>Hushåll</t>
         </is>
       </c>
-      <c r="G81" s="6" t="inlineStr">
-        <is>
-          <t>Matavfall</t>
-        </is>
-      </c>
+      <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="6" t="inlineStr">
         <is>
           <t>Behållarvolym</t>
@@ -27680,7 +27660,7 @@
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr">
@@ -27688,7 +27668,11 @@
           <t>matavfallspåsar</t>
         </is>
       </c>
-      <c r="M81" s="6" t="inlineStr"/>
+      <c r="M81" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -27713,11 +27697,7 @@
           <t>Hushåll</t>
         </is>
       </c>
-      <c r="G82" s="6" t="inlineStr">
-        <is>
-          <t>Matavfall</t>
-        </is>
-      </c>
+      <c r="G82" s="6" t="inlineStr"/>
       <c r="H82" s="6" t="inlineStr">
         <is>
           <t>Behållarvolym</t>
@@ -27735,7 +27715,7 @@
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr">
@@ -27743,7 +27723,11 @@
           <t>matavfallspåsar</t>
         </is>
       </c>
-      <c r="M82" s="6" t="inlineStr"/>
+      <c r="M82" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -27815,17 +27799,13 @@
           <t>Hushåll</t>
         </is>
       </c>
-      <c r="G84" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G84" s="6" t="inlineStr"/>
       <c r="H84" s="6" t="inlineStr"/>
       <c r="I84" s="6" t="inlineStr"/>
       <c r="J84" s="6" t="inlineStr"/>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L84" s="6" t="inlineStr">
@@ -27835,7 +27815,7 @@
       </c>
       <c r="M84" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -28285,7 +28265,7 @@
       </c>
       <c r="L93" s="6" t="inlineStr">
         <is>
-          <t>bad, disk, tvättbrunn, upp</t>
+          <t>bad-, disk-och, tvättbrunn, upp</t>
         </is>
       </c>
       <c r="M93" s="6" t="inlineStr">
@@ -28372,27 +28352,23 @@
           <t>Flerbostad/verksamhet</t>
         </is>
       </c>
-      <c r="G95" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G95" s="6" t="inlineStr"/>
       <c r="H95" s="6" t="inlineStr"/>
       <c r="I95" s="6" t="inlineStr"/>
       <c r="J95" s="6" t="inlineStr"/>
       <c r="K95" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L95" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>5-25, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M95" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -28419,27 +28395,23 @@
           <t>Flerbostad/verksamhet</t>
         </is>
       </c>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G96" s="6" t="inlineStr"/>
       <c r="H96" s="6" t="inlineStr"/>
       <c r="I96" s="6" t="inlineStr"/>
       <c r="J96" s="6" t="inlineStr"/>
       <c r="K96" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L96" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>25-35, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M96" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -28466,27 +28438,23 @@
           <t>Flerbostad/verksamhet</t>
         </is>
       </c>
-      <c r="G97" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G97" s="6" t="inlineStr"/>
       <c r="H97" s="6" t="inlineStr"/>
       <c r="I97" s="6" t="inlineStr"/>
       <c r="J97" s="6" t="inlineStr"/>
       <c r="K97" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L97" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>36-45, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M97" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -28513,27 +28481,23 @@
           <t>Flerbostad/verksamhet</t>
         </is>
       </c>
-      <c r="G98" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G98" s="6" t="inlineStr"/>
       <c r="H98" s="6" t="inlineStr"/>
       <c r="I98" s="6" t="inlineStr"/>
       <c r="J98" s="6" t="inlineStr"/>
       <c r="K98" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L98" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>46-55, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M98" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -28583,7 +28547,7 @@
       </c>
       <c r="L99" s="6" t="inlineStr">
         <is>
-          <t>brunnslock, hantering, kilogram, som, väger</t>
+          <t>15-25, brunnslock, hantering, kilogram, som, väger</t>
         </is>
       </c>
       <c r="M99" s="6" t="inlineStr">
@@ -28795,11 +28759,7 @@
           <t>Flerbostad/verksamhet</t>
         </is>
       </c>
-      <c r="G104" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G104" s="6" t="inlineStr"/>
       <c r="H104" s="6" t="inlineStr">
         <is>
           <t>Volym</t>
@@ -28813,7 +28773,7 @@
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L104" s="6" t="inlineStr">
@@ -28821,7 +28781,11 @@
           <t>brunn, budad, extra, ordinarie, samband, tank, tömning, upp</t>
         </is>
       </c>
-      <c r="M104" s="6" t="inlineStr"/>
+      <c r="M104" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
@@ -28857,7 +28821,7 @@
       </c>
       <c r="L105" s="6" t="inlineStr">
         <is>
-          <t>budning, inom, maj, oktober, ordinarie, tömningsperiod</t>
+          <t>budning, inom, maj-31, oktober, ordinarie, tömningsperiod</t>
         </is>
       </c>
       <c r="M105" s="6" t="inlineStr">
@@ -28900,7 +28864,7 @@
       </c>
       <c r="L106" s="6" t="inlineStr">
         <is>
-          <t>april, budning, nov, ordinarie, tömningsperiod, utanför</t>
+          <t>april, budning, nov-30, ordinarie, tömningsperiod, utanför</t>
         </is>
       </c>
       <c r="M106" s="6" t="inlineStr">
@@ -29124,7 +29088,7 @@
       </c>
       <c r="L110" s="6" t="inlineStr">
         <is>
-          <t>1000, 500, filtermassor, kilogram</t>
+          <t>500-1000, filtermassor, kilogram</t>
         </is>
       </c>
       <c r="M110" s="6" t="inlineStr">
@@ -29450,27 +29414,23 @@
           <t>Slam</t>
         </is>
       </c>
-      <c r="G117" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G117" s="6" t="inlineStr"/>
       <c r="H117" s="6" t="inlineStr"/>
       <c r="I117" s="6" t="inlineStr"/>
       <c r="J117" s="6" t="inlineStr"/>
       <c r="K117" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L117" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>5-25, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M117" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -29497,27 +29457,23 @@
           <t>Slam</t>
         </is>
       </c>
-      <c r="G118" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G118" s="6" t="inlineStr"/>
       <c r="H118" s="6" t="inlineStr"/>
       <c r="I118" s="6" t="inlineStr"/>
       <c r="J118" s="6" t="inlineStr"/>
       <c r="K118" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L118" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>25-35, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M118" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -29544,27 +29500,23 @@
           <t>Slam</t>
         </is>
       </c>
-      <c r="G119" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G119" s="6" t="inlineStr"/>
       <c r="H119" s="6" t="inlineStr"/>
       <c r="I119" s="6" t="inlineStr"/>
       <c r="J119" s="6" t="inlineStr"/>
       <c r="K119" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L119" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>36-45, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M119" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -29591,27 +29543,23 @@
           <t>Slam</t>
         </is>
       </c>
-      <c r="G120" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G120" s="6" t="inlineStr"/>
       <c r="H120" s="6" t="inlineStr"/>
       <c r="I120" s="6" t="inlineStr"/>
       <c r="J120" s="6" t="inlineStr"/>
       <c r="K120" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="L120" s="6" t="inlineStr">
         <is>
-          <t>dragning, extra, slang, vid</t>
+          <t>46-55, dragning, extra, slang, vid</t>
         </is>
       </c>
       <c r="M120" s="6" t="inlineStr">
         <is>
-          <t>Faktor kunde inte härledas från enhet/text.</t>
+          <t>Faktor kunde inte härledas från enhet/text. | Avfallstyp kunde inte härledas.</t>
         </is>
       </c>
     </row>
@@ -29661,7 +29609,7 @@
       </c>
       <c r="L121" s="6" t="inlineStr">
         <is>
-          <t>brunnslock, hantering, kilogram, som, väger</t>
+          <t>15-25, brunnslock, hantering, kilogram, som, väger</t>
         </is>
       </c>
       <c r="M121" s="6" t="inlineStr">
@@ -29916,11 +29864,7 @@
           <t>Slam</t>
         </is>
       </c>
-      <c r="G127" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G127" s="6" t="inlineStr"/>
       <c r="H127" s="6" t="inlineStr">
         <is>
           <t>Volym</t>
@@ -29934,7 +29878,7 @@
       </c>
       <c r="K127" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L127" s="6" t="inlineStr">
@@ -29942,7 +29886,11 @@
           <t>budad, extra, ordinarie, samband, tank, tömning, upp</t>
         </is>
       </c>
-      <c r="M127" s="6" t="inlineStr"/>
+      <c r="M127" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
@@ -29978,7 +29926,7 @@
       </c>
       <c r="L128" s="6" t="inlineStr">
         <is>
-          <t>budning, inom, maj, oktober, ordinarie, tömningsperiod</t>
+          <t>budning, inom, maj-31, oktober, ordinarie, tömningsperiod</t>
         </is>
       </c>
       <c r="M128" s="6" t="inlineStr">
@@ -30492,11 +30440,7 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G139" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G139" s="6" t="inlineStr"/>
       <c r="H139" s="6" t="inlineStr">
         <is>
           <t>Vikt</t>
@@ -30510,15 +30454,19 @@
       </c>
       <c r="K139" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L139" s="6" t="inlineStr">
         <is>
-          <t>kilogram, obehandlat, plastmatta, tapet, tjärpapp, träavfall</t>
-        </is>
-      </c>
-      <c r="M139" s="6" t="inlineStr"/>
+          <t>kilogram, plastmatta, tapet, tjärpapp, träavfall-obehandlat</t>
+        </is>
+      </c>
+      <c r="M139" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
@@ -30547,11 +30495,7 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G140" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G140" s="6" t="inlineStr"/>
       <c r="H140" s="6" t="inlineStr">
         <is>
           <t>Vikt</t>
@@ -30565,15 +30509,19 @@
       </c>
       <c r="K140" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L140" s="6" t="inlineStr">
         <is>
-          <t>behandlat, kilogram, plastmatta, tapet, tjärpapp, träavfall</t>
-        </is>
-      </c>
-      <c r="M140" s="6" t="inlineStr"/>
+          <t>kilogram, plastmatta, tapet, tjärpapp, träavfall-behandlat</t>
+        </is>
+      </c>
+      <c r="M140" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
@@ -30841,7 +30789,7 @@
       </c>
       <c r="L145" s="6" t="inlineStr">
         <is>
-          <t>fönster, karm, kilogram, planglas</t>
+          <t>fönster-och, karm, kilogram, planglas</t>
         </is>
       </c>
       <c r="M145" s="6" t="inlineStr">
@@ -31159,7 +31107,7 @@
       </c>
       <c r="L151" s="6" t="inlineStr">
         <is>
-          <t>stol, styck</t>
+          <t>styck, wc-stol</t>
         </is>
       </c>
       <c r="M151" s="6" t="inlineStr">
@@ -31652,7 +31600,7 @@
       </c>
       <c r="G161" s="6" t="inlineStr">
         <is>
-          <t>Farligt avfall</t>
+          <t>Elavfall</t>
         </is>
       </c>
       <c r="H161" s="6" t="inlineStr"/>
@@ -31811,7 +31759,11 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G164" s="6" t="inlineStr"/>
+      <c r="G164" s="6" t="inlineStr">
+        <is>
+          <t>Oljeavfall</t>
+        </is>
+      </c>
       <c r="H164" s="6" t="inlineStr">
         <is>
           <t>Vikt</t>
@@ -31825,7 +31777,7 @@
       </c>
       <c r="K164" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="L164" s="6" t="inlineStr">
@@ -31833,11 +31785,7 @@
           <t>förorenad, innehållande, kilogram, olja, pcb</t>
         </is>
       </c>
-      <c r="M164" s="6" t="inlineStr">
-        <is>
-          <t>Avfallstyp kunde inte härledas.</t>
-        </is>
-      </c>
+      <c r="M164" s="6" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
@@ -32361,11 +32309,7 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G174" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G174" s="6" t="inlineStr"/>
       <c r="H174" s="6" t="inlineStr">
         <is>
           <t>Vikt</t>
@@ -32379,7 +32323,7 @@
       </c>
       <c r="K174" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L174" s="6" t="inlineStr">
@@ -32387,7 +32331,11 @@
           <t>kilogram, kondensator, pcb, transformator</t>
         </is>
       </c>
-      <c r="M174" s="6" t="inlineStr"/>
+      <c r="M174" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="6" t="inlineStr">
@@ -33150,7 +33098,7 @@
       </c>
       <c r="L188" s="6" t="inlineStr">
         <is>
-          <t>haltiga, kilogram, småkemikalier</t>
+          <t>hg-haltiga, kilogram, småkemikalier</t>
         </is>
       </c>
       <c r="M188" s="6" t="inlineStr">
@@ -34451,7 +34399,11 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G212" s="6" t="inlineStr"/>
+      <c r="G212" s="6" t="inlineStr">
+        <is>
+          <t>Oljeavfall</t>
+        </is>
+      </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
           <t>Behållarvolym</t>
@@ -34465,7 +34417,7 @@
       </c>
       <c r="K212" s="6" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="L212" s="6" t="inlineStr">
@@ -34473,11 +34425,7 @@
           <t>förorenad, liter, olja, pcb</t>
         </is>
       </c>
-      <c r="M212" s="6" t="inlineStr">
-        <is>
-          <t>Avfallstyp kunde inte härledas.</t>
-        </is>
-      </c>
+      <c r="M212" s="6" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="6" t="inlineStr">
@@ -34525,7 +34473,7 @@
       </c>
       <c r="L213" s="6" t="inlineStr">
         <is>
-          <t>färg, kilogram, lack, limburkar, lösning</t>
+          <t>färg-, kilogram, lack-, limburkar, lösning</t>
         </is>
       </c>
       <c r="M213" s="6" t="inlineStr">
@@ -34580,7 +34528,7 @@
       </c>
       <c r="L214" s="6" t="inlineStr">
         <is>
-          <t>aerosoler, färg, kilogram, lack, limburkar, lösning</t>
+          <t>aerosoler, färg-, kilogram, lack-, limburkar, lösning</t>
         </is>
       </c>
       <c r="M214" s="6" t="inlineStr">
@@ -34690,7 +34638,7 @@
       </c>
       <c r="L216" s="6" t="inlineStr">
         <is>
-          <t>etylketonperoxid, härdare, kilogram, metyl</t>
+          <t>härdare, kilogram, metyl-etylketonperoxid</t>
         </is>
       </c>
       <c r="M216" s="6" t="inlineStr">
@@ -34800,7 +34748,7 @@
       </c>
       <c r="L218" s="6" t="inlineStr">
         <is>
-          <t>färg, kilogram, lack, limburkar, vattenbaserade</t>
+          <t>färg-, kilogram, lack-, limburkar, vattenbaserade</t>
         </is>
       </c>
       <c r="M218" s="6" t="inlineStr">
@@ -35276,11 +35224,7 @@
           <t>ÅVC/verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G227" s="6" t="inlineStr">
-        <is>
-          <t>Batterier</t>
-        </is>
-      </c>
+      <c r="G227" s="6" t="inlineStr"/>
       <c r="H227" s="6" t="inlineStr">
         <is>
           <t>Styck</t>
@@ -35294,15 +35238,19 @@
       </c>
       <c r="K227" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L227" s="6" t="inlineStr">
         <is>
-          <t>bil, bly, mcbatteri, styck</t>
-        </is>
-      </c>
-      <c r="M227" s="6" t="inlineStr"/>
+          <t>bil-, bly, mcbatteri, styck</t>
+        </is>
+      </c>
+      <c r="M227" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="6" t="inlineStr">
@@ -35519,7 +35467,7 @@
       </c>
       <c r="L231" s="6" t="inlineStr">
         <is>
-          <t>avfall, fast, installation, kilogram</t>
+          <t>el-avfall, fast, installation, kilogram</t>
         </is>
       </c>
       <c r="M231" s="6" t="inlineStr"/>
@@ -35574,7 +35522,7 @@
       </c>
       <c r="L232" s="6" t="inlineStr">
         <is>
-          <t>avfall, kabel, kilogram</t>
+          <t>el-avfall, kabel, kilogram</t>
         </is>
       </c>
       <c r="M232" s="6" t="inlineStr"/>
@@ -35739,7 +35687,7 @@
       </c>
       <c r="L235" s="6" t="inlineStr">
         <is>
-          <t>boxstyck, frysskåp, kyl</t>
+          <t>-boxstyck, frysskåp, kyl-</t>
         </is>
       </c>
       <c r="M235" s="6" t="inlineStr"/>
@@ -35794,7 +35742,7 @@
       </c>
       <c r="L236" s="6" t="inlineStr">
         <is>
-          <t>boxfrån, frysskåp, kilogram, kyl, verksamhet</t>
+          <t>-boxfrån, frysskåp, kilogram, kyl-, verksamhet</t>
         </is>
       </c>
       <c r="M236" s="6" t="inlineStr"/>
@@ -35845,7 +35793,7 @@
       </c>
       <c r="L237" s="6" t="inlineStr">
         <is>
-          <t>diskmaskin, spis, styck, tvätt</t>
+          <t>diskmaskin, spis, styck, tvätt-</t>
         </is>
       </c>
       <c r="M237" s="6" t="inlineStr">
@@ -35900,7 +35848,7 @@
       </c>
       <c r="L238" s="6" t="inlineStr">
         <is>
-          <t>diskmaskin, kilogram, spis, tvätt, verksamhet</t>
+          <t>diskmaskin, kilogram, spis, tvätt-, verksamhet</t>
         </is>
       </c>
       <c r="M238" s="6" t="inlineStr">
@@ -36254,11 +36202,7 @@
           <t>Verksamhetsavfall</t>
         </is>
       </c>
-      <c r="G245" s="6" t="inlineStr">
-        <is>
-          <t>Träavfall</t>
-        </is>
-      </c>
+      <c r="G245" s="6" t="inlineStr"/>
       <c r="H245" s="6" t="inlineStr">
         <is>
           <t>Tillfälle</t>
@@ -36272,7 +36216,7 @@
       </c>
       <c r="K245" s="6" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="L245" s="6" t="inlineStr">
@@ -36280,7 +36224,11 @@
           <t>administrativ, avfallsregistret, rapporteringsavgift, tillfälle</t>
         </is>
       </c>
-      <c r="M245" s="6" t="inlineStr"/>
+      <c r="M245" s="6" t="inlineStr">
+        <is>
+          <t>Avfallstyp kunde inte härledas.</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
@@ -36328,7 +36276,7 @@
       </c>
       <c r="L246" s="6" t="inlineStr">
         <is>
-          <t>avlämnarintyg, hämtplatsportalen, kretsen, ombud, registrering, tillfälle</t>
+          <t>avlämnarintyg, el-kretsen, hämtplatsportalen, ombud, registrering, tillfälle</t>
         </is>
       </c>
       <c r="M246" s="6" t="inlineStr">

</xml_diff>